<commit_message>
Improved raw data tab
</commit_message>
<xml_diff>
--- a/tmp/vaad/master_ledger.xlsx
+++ b/tmp/vaad/master_ledger.xlsx
@@ -14,6 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="April26" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="קופה קטנה" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="חוב דירה 13" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="תנועות מאי 2026" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191028" fullCalcOnLoad="1"/>
@@ -30,7 +31,7 @@
     <numFmt numFmtId="168" formatCode="_-&quot;₪&quot;* #,##0.00_-;\-&quot;₪&quot;* #,##0.00_-;_-&quot;₪&quot;* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="169" formatCode="_ [$₪-40D]\ * #,##0.00_ ;_ [$₪-40D]\ * \-#,##0.00_ ;_ [$₪-40D]\ * &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="23">
+  <fonts count="25">
     <font>
       <name val="Aptos Narrow"/>
       <family val="2"/>
@@ -191,8 +192,16 @@
       <u val="single"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="14">
+  <fills count="17">
     <fill>
       <patternFill/>
     </fill>
@@ -267,6 +276,21 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFFEB9C"/>
         <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002E4057"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D6F0D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
   </fills>
@@ -1046,7 +1070,7 @@
     <xf numFmtId="0" fontId="1" fillId="8" borderId="0"/>
     <xf numFmtId="168" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="241">
+  <cellXfs count="244">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="14" fontId="4" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="3"/>
@@ -1451,10 +1475,28 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="58" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
@@ -1467,26 +1509,8 @@
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment readingOrder="2"/>
@@ -1494,24 +1518,24 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="63" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="63" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="30" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="31" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="63" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="41" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="41" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="38" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="39" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="38" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="41" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="41" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="63" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment readingOrder="2"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
@@ -1538,6 +1562,15 @@
     <xf numFmtId="168" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="8"/>
     <xf numFmtId="169" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="168" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="23" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="9">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4544,7 +4577,7 @@
       </c>
       <c r="P46" s="29" t="n"/>
       <c r="Q46" s="33" t="n">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="S46" t="n">
         <v>4727351</v>
@@ -5050,10 +5083,10 @@
       <c r="H59" t="n">
         <v>350</v>
       </c>
+      <c r="I59" t="n">
+        <v>500</v>
+      </c>
       <c r="P59" s="131" t="n"/>
-      <c r="Q59" t="n">
-        <v>500</v>
-      </c>
       <c r="S59" t="n">
         <v>4660306</v>
       </c>
@@ -8664,41 +8697,41 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="205" t="inlineStr">
+      <c r="A1" s="196" t="inlineStr">
         <is>
           <t>בנק לאומי |</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="207" t="inlineStr">
+      <c r="A2" s="200" t="inlineStr">
         <is>
           <t>מס' חשבון : ‏‏ ‎885-37554/82‎</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="207" t="inlineStr">
+      <c r="A3" s="200" t="inlineStr">
         <is>
           <t>תאריך שמירה/הדפסה: 9/2/2026</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="208" t="n"/>
+      <c r="A4" s="202" t="n"/>
     </row>
     <row r="5" ht="15.75" customHeight="1" s="197">
-      <c r="A5" s="201" t="inlineStr">
+      <c r="A5" s="207" t="inlineStr">
         <is>
           <t>היתרה</t>
         </is>
       </c>
-      <c r="C5" s="200" t="inlineStr">
+      <c r="C5" s="206" t="inlineStr">
         <is>
           <t>מסגרת האשראי</t>
         </is>
       </c>
-      <c r="E5" s="206" t="inlineStr">
+      <c r="E5" s="198" t="inlineStr">
         <is>
           <t>נכון לתאריך</t>
         </is>
@@ -8708,25 +8741,25 @@
       <c r="I5" s="148" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="207" t="n"/>
-      <c r="C6" s="202" t="n"/>
-      <c r="E6" s="199" t="n"/>
+      <c r="A6" s="200" t="n"/>
+      <c r="C6" s="203" t="n"/>
+      <c r="E6" s="205" t="n"/>
       <c r="G6" s="148" t="n"/>
       <c r="H6" s="148" t="n"/>
       <c r="I6" s="148" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="204" t="inlineStr">
+      <c r="A7" s="201" t="inlineStr">
         <is>
           <t>₪ 22,270.89</t>
         </is>
       </c>
-      <c r="C7" s="203" t="inlineStr">
+      <c r="C7" s="208" t="inlineStr">
         <is>
           <t>₪ 0.00</t>
         </is>
       </c>
-      <c r="E7" s="198" t="inlineStr">
+      <c r="E7" s="204" t="inlineStr">
         <is>
           <t>09.02.26</t>
         </is>
@@ -8736,22 +8769,22 @@
       <c r="I7" s="148" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="204" t="inlineStr">
+      <c r="A8" s="201" t="inlineStr">
         <is>
           <t>* כולל תנועות היום</t>
         </is>
       </c>
-      <c r="C8" s="202" t="n"/>
-      <c r="E8" s="199" t="n"/>
+      <c r="C8" s="203" t="n"/>
+      <c r="E8" s="205" t="n"/>
       <c r="G8" s="148" t="n"/>
       <c r="H8" s="148" t="n"/>
       <c r="I8" s="148" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="196" t="n"/>
+      <c r="A9" s="199" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="196" t="n"/>
+      <c r="A10" s="199" t="n"/>
     </row>
     <row r="11" customFormat="1" s="4">
       <c r="A11" s="2" t="n">
@@ -11165,14 +11198,14 @@
     </row>
   </sheetData>
   <mergeCells count="18">
-    <mergeCell ref="A6:B6"/>
     <mergeCell ref="E6:F6"/>
     <mergeCell ref="C6:D6"/>
-    <mergeCell ref="A2:I2"/>
     <mergeCell ref="C7:D7"/>
+    <mergeCell ref="A7:B7"/>
     <mergeCell ref="A10:I10"/>
     <mergeCell ref="E7:F7"/>
-    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="A2:I2"/>
+    <mergeCell ref="E8:F8"/>
     <mergeCell ref="C5:D5"/>
     <mergeCell ref="A5:B5"/>
     <mergeCell ref="A1:I1"/>
@@ -11181,7 +11214,7 @@
     <mergeCell ref="A3:I3"/>
     <mergeCell ref="A8:B8"/>
     <mergeCell ref="A4:I4"/>
-    <mergeCell ref="E8:F8"/>
+    <mergeCell ref="A6:B6"/>
     <mergeCell ref="C8:D8"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -13551,8 +13584,8 @@
     <mergeCell ref="E5:F5"/>
     <mergeCell ref="A3:I3"/>
     <mergeCell ref="A12:I12"/>
+    <mergeCell ref="A6:B6"/>
     <mergeCell ref="E8:F8"/>
-    <mergeCell ref="A6:B6"/>
     <mergeCell ref="A2:I2"/>
     <mergeCell ref="A7:B7"/>
     <mergeCell ref="A4:I4"/>
@@ -16655,7 +16688,7 @@
       <c r="V11" s="47" t="n"/>
     </row>
     <row r="12" ht="18.75" customHeight="1" s="197">
-      <c r="A12" s="211" t="inlineStr">
+      <c r="A12" s="214" t="inlineStr">
         <is>
           <t xml:space="preserve"> חוב שנת 2020</t>
         </is>
@@ -16746,10 +16779,10 @@
       <c r="V13" s="47" t="n"/>
     </row>
     <row r="14" ht="15.75" customHeight="1" s="197">
-      <c r="A14" s="214" t="n">
+      <c r="A14" s="218" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="217" t="inlineStr">
+      <c r="B14" s="215" t="inlineStr">
         <is>
           <t>בכר</t>
         </is>
@@ -16804,8 +16837,8 @@
       <c r="V14" s="47" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="215" t="n"/>
-      <c r="B15" s="218" t="n"/>
+      <c r="A15" s="219" t="n"/>
+      <c r="B15" s="216" t="n"/>
       <c r="C15" s="58" t="n">
         <v>500</v>
       </c>
@@ -16842,8 +16875,8 @@
       <c r="V15" s="47" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="216" t="n"/>
-      <c r="B16" s="219" t="n"/>
+      <c r="A16" s="220" t="n"/>
+      <c r="B16" s="217" t="n"/>
       <c r="C16" s="50" t="inlineStr">
         <is>
           <t>טרם שולם</t>
@@ -16918,7 +16951,7 @@
       <c r="V17" s="47" t="n"/>
     </row>
     <row r="18" ht="18.75" customHeight="1" s="197">
-      <c r="A18" s="211" t="inlineStr">
+      <c r="A18" s="214" t="inlineStr">
         <is>
           <t>חוב שנת 2021</t>
         </is>
@@ -17037,10 +17070,10 @@
       <c r="V19" s="47" t="n"/>
     </row>
     <row r="20" ht="15.75" customHeight="1" s="197">
-      <c r="A20" s="214" t="n">
+      <c r="A20" s="218" t="n">
         <v>13</v>
       </c>
-      <c r="B20" s="217" t="inlineStr">
+      <c r="B20" s="215" t="inlineStr">
         <is>
           <t>בכר</t>
         </is>
@@ -17119,8 +17152,8 @@
       <c r="V20" s="47" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="215" t="n"/>
-      <c r="B21" s="218" t="n"/>
+      <c r="A21" s="219" t="n"/>
+      <c r="B21" s="216" t="n"/>
       <c r="C21" s="60" t="n">
         <v>320</v>
       </c>
@@ -17169,8 +17202,8 @@
       <c r="V21" s="47" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="216" t="n"/>
-      <c r="B22" s="219" t="n"/>
+      <c r="A22" s="220" t="n"/>
+      <c r="B22" s="217" t="n"/>
       <c r="C22" s="63" t="inlineStr">
         <is>
           <t>שולם</t>
@@ -17269,7 +17302,7 @@
       <c r="V23" s="47" t="n"/>
     </row>
     <row r="24" ht="18.75" customHeight="1" s="197">
-      <c r="A24" s="211" t="inlineStr">
+      <c r="A24" s="214" t="inlineStr">
         <is>
           <t xml:space="preserve"> חוב שנת 2022</t>
         </is>
@@ -17378,10 +17411,10 @@
       <c r="V25" s="47" t="n"/>
     </row>
     <row r="26" ht="15.75" customHeight="1" s="197">
-      <c r="A26" s="214" t="n">
+      <c r="A26" s="218" t="n">
         <v>13</v>
       </c>
-      <c r="B26" s="217" t="inlineStr">
+      <c r="B26" s="215" t="inlineStr">
         <is>
           <t>בכר</t>
         </is>
@@ -17456,8 +17489,8 @@
       <c r="V26" s="47" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="215" t="n"/>
-      <c r="B27" s="218" t="n"/>
+      <c r="A27" s="219" t="n"/>
+      <c r="B27" s="216" t="n"/>
       <c r="C27" s="71" t="n">
         <v>320</v>
       </c>
@@ -17504,8 +17537,8 @@
       <c r="V27" s="47" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="216" t="n"/>
-      <c r="B28" s="219" t="n"/>
+      <c r="A28" s="220" t="n"/>
+      <c r="B28" s="217" t="n"/>
       <c r="C28" s="74" t="inlineStr">
         <is>
           <t>טרם שולם</t>
@@ -17600,7 +17633,7 @@
       <c r="V29" s="47" t="n"/>
     </row>
     <row r="30" ht="18.75" customHeight="1" s="197">
-      <c r="A30" s="211" t="inlineStr">
+      <c r="A30" s="214" t="inlineStr">
         <is>
           <t xml:space="preserve">חוב שנת 2023 </t>
         </is>
@@ -17709,10 +17742,10 @@
       <c r="V31" s="47" t="n"/>
     </row>
     <row r="32" ht="15.75" customHeight="1" s="197">
-      <c r="A32" s="214" t="n">
+      <c r="A32" s="218" t="n">
         <v>13</v>
       </c>
-      <c r="B32" s="217" t="inlineStr">
+      <c r="B32" s="215" t="inlineStr">
         <is>
           <t>בכר</t>
         </is>
@@ -17787,8 +17820,8 @@
       <c r="V32" s="47" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="215" t="n"/>
-      <c r="B33" s="218" t="n"/>
+      <c r="A33" s="219" t="n"/>
+      <c r="B33" s="216" t="n"/>
       <c r="C33" s="83" t="n">
         <v>320</v>
       </c>
@@ -17835,8 +17868,8 @@
       <c r="V33" s="47" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="216" t="n"/>
-      <c r="B34" s="219" t="n"/>
+      <c r="A34" s="220" t="n"/>
+      <c r="B34" s="217" t="n"/>
       <c r="C34" s="84" t="inlineStr">
         <is>
           <t>טרם שולם</t>
@@ -17931,7 +17964,7 @@
       <c r="V35" s="47" t="n"/>
     </row>
     <row r="36" ht="18.75" customHeight="1" s="197">
-      <c r="A36" s="211" t="inlineStr">
+      <c r="A36" s="214" t="inlineStr">
         <is>
           <t xml:space="preserve">שנת 2024 </t>
         </is>
@@ -18045,10 +18078,10 @@
       <c r="V37" s="47" t="n"/>
     </row>
     <row r="38" ht="15.75" customHeight="1" s="197">
-      <c r="A38" s="214" t="n">
+      <c r="A38" s="218" t="n">
         <v>13</v>
       </c>
-      <c r="B38" s="217" t="inlineStr">
+      <c r="B38" s="215" t="inlineStr">
         <is>
           <t>בכר</t>
         </is>
@@ -18127,8 +18160,8 @@
       <c r="V38" s="47" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="215" t="n"/>
-      <c r="B39" s="218" t="n"/>
+      <c r="A39" s="219" t="n"/>
+      <c r="B39" s="216" t="n"/>
       <c r="C39" s="60" t="n">
         <v>320</v>
       </c>
@@ -18177,8 +18210,8 @@
       <c r="V39" s="47" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="216" t="n"/>
-      <c r="B40" s="219" t="n"/>
+      <c r="A40" s="220" t="n"/>
+      <c r="B40" s="217" t="n"/>
       <c r="C40" s="63" t="inlineStr">
         <is>
           <t>שולם</t>
@@ -18279,7 +18312,7 @@
     <row r="42">
       <c r="A42" s="47" t="n"/>
       <c r="B42" s="47" t="n"/>
-      <c r="C42" s="220" t="inlineStr">
+      <c r="C42" s="211" t="inlineStr">
         <is>
           <t>סיכום</t>
         </is>
@@ -20634,25 +20667,25 @@
     <mergeCell ref="E68:F68"/>
     <mergeCell ref="A75:I75"/>
     <mergeCell ref="A24:N24"/>
-    <mergeCell ref="A89:I89"/>
-    <mergeCell ref="E71:F71"/>
     <mergeCell ref="A30:N30"/>
     <mergeCell ref="A20:A22"/>
     <mergeCell ref="A66:I66"/>
+    <mergeCell ref="A89:I89"/>
+    <mergeCell ref="E71:F71"/>
+    <mergeCell ref="A32:A34"/>
+    <mergeCell ref="A38:A40"/>
+    <mergeCell ref="A14:A16"/>
+    <mergeCell ref="A12:I12"/>
     <mergeCell ref="A94:B94"/>
+    <mergeCell ref="A36:N36"/>
     <mergeCell ref="A74:I74"/>
     <mergeCell ref="A70:B70"/>
+    <mergeCell ref="A69:B69"/>
     <mergeCell ref="E92:F92"/>
-    <mergeCell ref="A12:I12"/>
-    <mergeCell ref="A14:A16"/>
-    <mergeCell ref="A38:A40"/>
-    <mergeCell ref="A32:A34"/>
-    <mergeCell ref="A69:B69"/>
-    <mergeCell ref="A36:N36"/>
     <mergeCell ref="A95:I95"/>
+    <mergeCell ref="B20:B22"/>
     <mergeCell ref="C94:D94"/>
     <mergeCell ref="B26:B28"/>
-    <mergeCell ref="B20:B22"/>
     <mergeCell ref="E94:F94"/>
     <mergeCell ref="C93:D93"/>
     <mergeCell ref="E69:F69"/>
@@ -20674,13 +20707,2447 @@
     <mergeCell ref="C42:H42"/>
     <mergeCell ref="A68:B68"/>
     <mergeCell ref="A88:I88"/>
+    <mergeCell ref="B14:B16"/>
     <mergeCell ref="A93:B93"/>
-    <mergeCell ref="B14:B16"/>
+    <mergeCell ref="B38:B40"/>
     <mergeCell ref="E93:F93"/>
-    <mergeCell ref="B38:B40"/>
     <mergeCell ref="A87:I87"/>
     <mergeCell ref="C69:D69"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M43"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" style="197" min="1" max="1"/>
+    <col width="10" customWidth="1" style="197" min="2" max="2"/>
+    <col width="18" customWidth="1" style="197" min="3" max="3"/>
+    <col width="12" customWidth="1" style="197" min="4" max="4"/>
+    <col width="10" customWidth="1" style="197" min="5" max="5"/>
+    <col width="22" customWidth="1" style="197" min="6" max="6"/>
+    <col width="7" customWidth="1" style="197" min="7" max="7"/>
+    <col width="20" customWidth="1" style="197" min="8" max="8"/>
+    <col width="18" customWidth="1" style="197" min="9" max="9"/>
+    <col width="12" customWidth="1" style="197" min="10" max="10"/>
+    <col width="14" customWidth="1" style="197" min="11" max="11"/>
+    <col width="20" customWidth="1" style="197" min="12" max="12"/>
+    <col width="50" customWidth="1" style="197" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1" s="197">
+      <c r="A1" s="241" t="inlineStr">
+        <is>
+          <t>תאריך</t>
+        </is>
+      </c>
+      <c r="B1" s="241" t="inlineStr">
+        <is>
+          <t>כניסה/יציאה</t>
+        </is>
+      </c>
+      <c r="C1" s="241" t="inlineStr">
+        <is>
+          <t>תיאור</t>
+        </is>
+      </c>
+      <c r="D1" s="241" t="inlineStr">
+        <is>
+          <t>אסמכתא</t>
+        </is>
+      </c>
+      <c r="E1" s="241" t="inlineStr">
+        <is>
+          <t>סכום (₪)</t>
+        </is>
+      </c>
+      <c r="F1" s="241" t="inlineStr">
+        <is>
+          <t>שם שולח / ישות</t>
+        </is>
+      </c>
+      <c r="G1" s="241" t="inlineStr">
+        <is>
+          <t>דירה</t>
+        </is>
+      </c>
+      <c r="H1" s="241" t="inlineStr">
+        <is>
+          <t>דייר</t>
+        </is>
+      </c>
+      <c r="I1" s="241" t="inlineStr">
+        <is>
+          <t>קטגוריה</t>
+        </is>
+      </c>
+      <c r="J1" s="241" t="inlineStr">
+        <is>
+          <t>חודש תשלום</t>
+        </is>
+      </c>
+      <c r="K1" s="241" t="inlineStr">
+        <is>
+          <t>שיטת התאמה</t>
+        </is>
+      </c>
+      <c r="L1" s="241" t="inlineStr">
+        <is>
+          <t>הערות</t>
+        </is>
+      </c>
+      <c r="M1" s="241" t="inlineStr">
+        <is>
+          <t>תאור מורחב</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="16" customHeight="1" s="197">
+      <c r="A2" s="242" t="inlineStr">
+        <is>
+          <t>11/05/2026</t>
+        </is>
+      </c>
+      <c r="B2" s="242" t="inlineStr">
+        <is>
+          <t>הכנסה ✅</t>
+        </is>
+      </c>
+      <c r="C2" s="242" t="inlineStr">
+        <is>
+          <t>הוראת קבע</t>
+        </is>
+      </c>
+      <c r="D2" s="242" t="inlineStr">
+        <is>
+          <t>974656</t>
+        </is>
+      </c>
+      <c r="E2" s="242" t="n">
+        <v>350</v>
+      </c>
+      <c r="F2" s="242" t="inlineStr"/>
+      <c r="G2" s="242" t="inlineStr"/>
+      <c r="H2" s="242" t="inlineStr"/>
+      <c r="I2" s="242" t="inlineStr"/>
+      <c r="J2" s="242" t="inlineStr">
+        <is>
+          <t>05/2026</t>
+        </is>
+      </c>
+      <c r="K2" s="242" t="inlineStr"/>
+      <c r="L2" s="242" t="inlineStr"/>
+      <c r="M2" s="242" t="inlineStr"/>
+    </row>
+    <row r="3" ht="16" customHeight="1" s="197">
+      <c r="A3" s="242" t="inlineStr">
+        <is>
+          <t>11/05/2026</t>
+        </is>
+      </c>
+      <c r="B3" s="242" t="inlineStr">
+        <is>
+          <t>הכנסה ✅</t>
+        </is>
+      </c>
+      <c r="C3" s="242" t="inlineStr">
+        <is>
+          <t>העברה דיגיטל</t>
+        </is>
+      </c>
+      <c r="D3" s="242" t="inlineStr">
+        <is>
+          <t>699219459</t>
+        </is>
+      </c>
+      <c r="E3" s="242" t="n">
+        <v>500</v>
+      </c>
+      <c r="F3" s="242" t="inlineStr">
+        <is>
+          <t>אליאס סמעאן</t>
+        </is>
+      </c>
+      <c r="G3" s="242" t="inlineStr">
+        <is>
+          <t>58</t>
+        </is>
+      </c>
+      <c r="H3" s="242" t="inlineStr">
+        <is>
+          <t>סמעאן</t>
+        </is>
+      </c>
+      <c r="I3" s="242" t="inlineStr"/>
+      <c r="J3" s="242" t="inlineStr">
+        <is>
+          <t>05/2026</t>
+        </is>
+      </c>
+      <c r="K3" s="242" t="inlineStr">
+        <is>
+          <t>fuzzy_name</t>
+        </is>
+      </c>
+      <c r="L3" s="242" t="inlineStr">
+        <is>
+          <t>⚠️ צפוי ₪350 | בדיקה ידנית</t>
+        </is>
+      </c>
+      <c r="M3" s="242" t="inlineStr">
+        <is>
+          <t>העברה מאת: אליאס סמעאן 10-877-003268585 קופה קטנה</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="16" customHeight="1" s="197">
+      <c r="A4" s="243" t="inlineStr">
+        <is>
+          <t>01/05/2026</t>
+        </is>
+      </c>
+      <c r="B4" s="243" t="inlineStr">
+        <is>
+          <t>הוצאה 💸</t>
+        </is>
+      </c>
+      <c r="C4" s="243" t="inlineStr">
+        <is>
+          <t>נובולה בע"מ-י</t>
+        </is>
+      </c>
+      <c r="D4" s="243" t="inlineStr">
+        <is>
+          <t>42663</t>
+        </is>
+      </c>
+      <c r="E4" s="243" t="n">
+        <v>77</v>
+      </c>
+      <c r="F4" s="243" t="inlineStr">
+        <is>
+          <t>נובולה</t>
+        </is>
+      </c>
+      <c r="G4" s="243" t="inlineStr"/>
+      <c r="H4" s="243" t="inlineStr"/>
+      <c r="I4" s="243" t="inlineStr">
+        <is>
+          <t>Novula - מסך טלויזיה</t>
+        </is>
+      </c>
+      <c r="J4" s="243" t="inlineStr">
+        <is>
+          <t>05/2026</t>
+        </is>
+      </c>
+      <c r="K4" s="243" t="inlineStr"/>
+      <c r="L4" s="243" t="inlineStr"/>
+      <c r="M4" s="243" t="inlineStr"/>
+    </row>
+    <row r="5" ht="16" customHeight="1" s="197">
+      <c r="A5" s="242" t="inlineStr">
+        <is>
+          <t>01/05/2026</t>
+        </is>
+      </c>
+      <c r="B5" s="242" t="inlineStr">
+        <is>
+          <t>הכנסה ✅</t>
+        </is>
+      </c>
+      <c r="C5" s="242" t="inlineStr">
+        <is>
+          <t>בנק הפועלים</t>
+        </is>
+      </c>
+      <c r="D5" s="242" t="inlineStr">
+        <is>
+          <t>99012</t>
+        </is>
+      </c>
+      <c r="E5" s="242" t="n">
+        <v>320</v>
+      </c>
+      <c r="F5" s="242" t="inlineStr">
+        <is>
+          <t>ברייב יולי</t>
+        </is>
+      </c>
+      <c r="G5" s="242" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="H5" s="242" t="inlineStr">
+        <is>
+          <t>ברייב יולי</t>
+        </is>
+      </c>
+      <c r="I5" s="242" t="inlineStr"/>
+      <c r="J5" s="242" t="inlineStr">
+        <is>
+          <t>05/2026</t>
+        </is>
+      </c>
+      <c r="K5" s="242" t="inlineStr">
+        <is>
+          <t>fuzzy_name</t>
+        </is>
+      </c>
+      <c r="L5" s="242" t="inlineStr">
+        <is>
+          <t>⚠️ צפוי ₪350 | בדיקה ידנית</t>
+        </is>
+      </c>
+      <c r="M5" s="242" t="inlineStr">
+        <is>
+          <t>העברה מאת: ברייב יולי 12-701-000404014 ועד בית</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="16" customHeight="1" s="197">
+      <c r="A6" s="242" t="inlineStr">
+        <is>
+          <t>01/05/2026</t>
+        </is>
+      </c>
+      <c r="B6" s="242" t="inlineStr">
+        <is>
+          <t>הכנסה ✅</t>
+        </is>
+      </c>
+      <c r="C6" s="242" t="inlineStr">
+        <is>
+          <t>בנק הפועלים</t>
+        </is>
+      </c>
+      <c r="D6" s="242" t="inlineStr">
+        <is>
+          <t>99012</t>
+        </is>
+      </c>
+      <c r="E6" s="242" t="n">
+        <v>350</v>
+      </c>
+      <c r="F6" s="242" t="inlineStr">
+        <is>
+          <t>רועי ולי-ש</t>
+        </is>
+      </c>
+      <c r="G6" s="242" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
+      <c r="H6" s="242" t="inlineStr">
+        <is>
+          <t>רועי ולי</t>
+        </is>
+      </c>
+      <c r="I6" s="242" t="inlineStr"/>
+      <c r="J6" s="242" t="inlineStr">
+        <is>
+          <t>05/2026</t>
+        </is>
+      </c>
+      <c r="K6" s="242" t="inlineStr">
+        <is>
+          <t>fuzzy_name</t>
+        </is>
+      </c>
+      <c r="L6" s="242" t="inlineStr"/>
+      <c r="M6" s="242" t="inlineStr">
+        <is>
+          <t>העברה מאת: רועי ולי-ש 12-700-000616685 ועד בית</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="16" customHeight="1" s="197">
+      <c r="A7" s="242" t="inlineStr">
+        <is>
+          <t>01/05/2026</t>
+        </is>
+      </c>
+      <c r="B7" s="242" t="inlineStr">
+        <is>
+          <t>הכנסה ✅</t>
+        </is>
+      </c>
+      <c r="C7" s="242" t="inlineStr">
+        <is>
+          <t>בנק הפועלים</t>
+        </is>
+      </c>
+      <c r="D7" s="242" t="inlineStr">
+        <is>
+          <t>99012</t>
+        </is>
+      </c>
+      <c r="E7" s="242" t="n">
+        <v>350</v>
+      </c>
+      <c r="F7" s="242" t="inlineStr">
+        <is>
+          <t>מנגיסטו דג</t>
+        </is>
+      </c>
+      <c r="G7" s="242" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H7" s="242" t="inlineStr">
+        <is>
+          <t>מנגיסטו</t>
+        </is>
+      </c>
+      <c r="I7" s="242" t="inlineStr"/>
+      <c r="J7" s="242" t="inlineStr">
+        <is>
+          <t>05/2026</t>
+        </is>
+      </c>
+      <c r="K7" s="242" t="inlineStr">
+        <is>
+          <t>fuzzy_name</t>
+        </is>
+      </c>
+      <c r="L7" s="242" t="inlineStr"/>
+      <c r="M7" s="242" t="inlineStr">
+        <is>
+          <t>העברה מאת: מנגיסטו דג 12-703-000091338 לוועד הבית</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="16" customHeight="1" s="197">
+      <c r="A8" s="242" t="inlineStr">
+        <is>
+          <t>01/05/2026</t>
+        </is>
+      </c>
+      <c r="B8" s="242" t="inlineStr">
+        <is>
+          <t>הכנסה ✅</t>
+        </is>
+      </c>
+      <c r="C8" s="242" t="inlineStr">
+        <is>
+          <t>הוראת קבע</t>
+        </is>
+      </c>
+      <c r="D8" s="242" t="inlineStr">
+        <is>
+          <t>4873628</t>
+        </is>
+      </c>
+      <c r="E8" s="242" t="n">
+        <v>350</v>
+      </c>
+      <c r="F8" s="242" t="inlineStr">
+        <is>
+          <t>אליזבט בינשטוק</t>
+        </is>
+      </c>
+      <c r="G8" s="242" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="H8" s="242" t="inlineStr">
+        <is>
+          <t>אליזבט בינשטוק</t>
+        </is>
+      </c>
+      <c r="I8" s="242" t="inlineStr"/>
+      <c r="J8" s="242" t="inlineStr">
+        <is>
+          <t>05/2026</t>
+        </is>
+      </c>
+      <c r="K8" s="242" t="inlineStr">
+        <is>
+          <t>fuzzy_name</t>
+        </is>
+      </c>
+      <c r="L8" s="242" t="inlineStr"/>
+      <c r="M8" s="242" t="inlineStr">
+        <is>
+          <t>העברה מאת: אליזבט בינשטוק, 10-891-003641132 תשלום בהוראת קבע</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="16" customHeight="1" s="197">
+      <c r="A9" s="243" t="inlineStr">
+        <is>
+          <t>01/05/2026</t>
+        </is>
+      </c>
+      <c r="B9" s="243" t="inlineStr">
+        <is>
+          <t>הוצאה 💸</t>
+        </is>
+      </c>
+      <c r="C9" s="243" t="inlineStr">
+        <is>
+          <t>מסלול מורחב</t>
+        </is>
+      </c>
+      <c r="D9" s="243" t="inlineStr">
+        <is>
+          <t>13578</t>
+        </is>
+      </c>
+      <c r="E9" s="243" t="n">
+        <v>25</v>
+      </c>
+      <c r="F9" s="243" t="inlineStr">
+        <is>
+          <t>בנק</t>
+        </is>
+      </c>
+      <c r="G9" s="243" t="inlineStr"/>
+      <c r="H9" s="243" t="inlineStr"/>
+      <c r="I9" s="243" t="inlineStr">
+        <is>
+          <t>מסלול בנק</t>
+        </is>
+      </c>
+      <c r="J9" s="243" t="inlineStr">
+        <is>
+          <t>05/2026</t>
+        </is>
+      </c>
+      <c r="K9" s="243" t="inlineStr"/>
+      <c r="L9" s="243" t="inlineStr"/>
+      <c r="M9" s="243" t="inlineStr"/>
+    </row>
+    <row r="10" ht="16" customHeight="1" s="197">
+      <c r="A10" s="243" t="inlineStr">
+        <is>
+          <t>01/05/2026</t>
+        </is>
+      </c>
+      <c r="B10" s="243" t="inlineStr">
+        <is>
+          <t>הוצאה 💸</t>
+        </is>
+      </c>
+      <c r="C10" s="243" t="inlineStr">
+        <is>
+          <t>עמל.ערוץ יש 12</t>
+        </is>
+      </c>
+      <c r="D10" s="243" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="E10" s="243" t="n">
+        <v>19.8</v>
+      </c>
+      <c r="F10" s="243" t="inlineStr">
+        <is>
+          <t>בנק</t>
+        </is>
+      </c>
+      <c r="G10" s="243" t="inlineStr"/>
+      <c r="H10" s="243" t="inlineStr"/>
+      <c r="I10" s="243" t="inlineStr">
+        <is>
+          <t>עמלות בנק</t>
+        </is>
+      </c>
+      <c r="J10" s="243" t="inlineStr">
+        <is>
+          <t>05/2026</t>
+        </is>
+      </c>
+      <c r="K10" s="243" t="inlineStr"/>
+      <c r="L10" s="243" t="inlineStr"/>
+      <c r="M10" s="243" t="inlineStr">
+        <is>
+          <t>סכום החיוב מייצג את מספר התנועות שבוצעו בערוץ ישיר/פקיד.  מספר התנועות מופיע בסמוך למלל.  סכום העמלה לפעולה הינו כפי המופיע בתעריף העמלות ליחיד/תאגיד ובהתאם להטבות הקיימות ללקוח דהיינו סכום חיוב = מספר תנועות ערוץ פקיד/ישיר כפול תעריף העמלה בחשבון הלקוח</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="16" customHeight="1" s="197">
+      <c r="A11" s="242" t="inlineStr">
+        <is>
+          <t>03/05/2026</t>
+        </is>
+      </c>
+      <c r="B11" s="242" t="inlineStr">
+        <is>
+          <t>הכנסה ✅</t>
+        </is>
+      </c>
+      <c r="C11" s="242" t="inlineStr">
+        <is>
+          <t>הוראת קבע</t>
+        </is>
+      </c>
+      <c r="D11" s="242" t="inlineStr">
+        <is>
+          <t>4668970</t>
+        </is>
+      </c>
+      <c r="E11" s="242" t="n">
+        <v>350</v>
+      </c>
+      <c r="F11" s="242" t="inlineStr">
+        <is>
+          <t>פריידמן נטליה</t>
+        </is>
+      </c>
+      <c r="G11" s="242" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="H11" s="242" t="inlineStr">
+        <is>
+          <t>פריידמן נטליה</t>
+        </is>
+      </c>
+      <c r="I11" s="242" t="inlineStr"/>
+      <c r="J11" s="242" t="inlineStr">
+        <is>
+          <t>05/2026</t>
+        </is>
+      </c>
+      <c r="K11" s="242" t="inlineStr">
+        <is>
+          <t>fuzzy_name</t>
+        </is>
+      </c>
+      <c r="L11" s="242" t="inlineStr"/>
+      <c r="M11" s="242" t="inlineStr">
+        <is>
+          <t>העברה מאת: פריידמן נטליה 10-882-044876260 תשלום</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="16" customHeight="1" s="197">
+      <c r="A12" s="242" t="inlineStr">
+        <is>
+          <t>03/05/2026</t>
+        </is>
+      </c>
+      <c r="B12" s="242" t="inlineStr">
+        <is>
+          <t>הכנסה ✅</t>
+        </is>
+      </c>
+      <c r="C12" s="242" t="inlineStr">
+        <is>
+          <t>הוראת קבע</t>
+        </is>
+      </c>
+      <c r="D12" s="242" t="inlineStr">
+        <is>
+          <t>4878373</t>
+        </is>
+      </c>
+      <c r="E12" s="242" t="n">
+        <v>350</v>
+      </c>
+      <c r="F12" s="242" t="inlineStr">
+        <is>
+          <t>גל ברזני, שני ול</t>
+        </is>
+      </c>
+      <c r="G12" s="242" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="H12" s="242" t="inlineStr">
+        <is>
+          <t>נחשון</t>
+        </is>
+      </c>
+      <c r="I12" s="242" t="inlineStr"/>
+      <c r="J12" s="242" t="inlineStr">
+        <is>
+          <t>05/2026</t>
+        </is>
+      </c>
+      <c r="K12" s="242" t="inlineStr">
+        <is>
+          <t>apt_hint</t>
+        </is>
+      </c>
+      <c r="L12" s="242" t="inlineStr"/>
+      <c r="M12" s="242" t="inlineStr">
+        <is>
+          <t>העברה מאת: גל ברזני, שני ול 10-635-001111123 וועד בית דירה 56</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="16" customHeight="1" s="197">
+      <c r="A13" s="242" t="inlineStr">
+        <is>
+          <t>04/05/2026</t>
+        </is>
+      </c>
+      <c r="B13" s="242" t="inlineStr">
+        <is>
+          <t>הכנסה ✅</t>
+        </is>
+      </c>
+      <c r="C13" s="242" t="inlineStr">
+        <is>
+          <t>בנק הפועלים</t>
+        </is>
+      </c>
+      <c r="D13" s="242" t="inlineStr">
+        <is>
+          <t>99012</t>
+        </is>
+      </c>
+      <c r="E13" s="242" t="n">
+        <v>350</v>
+      </c>
+      <c r="F13" s="242" t="inlineStr">
+        <is>
+          <t>גואטה מררו אורית</t>
+        </is>
+      </c>
+      <c r="G13" s="242" t="inlineStr">
+        <is>
+          <t>37</t>
+        </is>
+      </c>
+      <c r="H13" s="242" t="inlineStr">
+        <is>
+          <t>חיון</t>
+        </is>
+      </c>
+      <c r="I13" s="242" t="inlineStr"/>
+      <c r="J13" s="242" t="inlineStr">
+        <is>
+          <t>04/2026</t>
+        </is>
+      </c>
+      <c r="K13" s="242" t="inlineStr">
+        <is>
+          <t>fuzzy_name</t>
+        </is>
+      </c>
+      <c r="L13" s="242" t="inlineStr"/>
+      <c r="M13" s="242" t="inlineStr">
+        <is>
+          <t>העברה מאת: גואטה מררו אורית 12-704-000515151 ועד בית אפריל</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="16" customHeight="1" s="197">
+      <c r="A14" s="242" t="inlineStr">
+        <is>
+          <t>04/05/2026</t>
+        </is>
+      </c>
+      <c r="B14" s="242" t="inlineStr">
+        <is>
+          <t>הכנסה ✅</t>
+        </is>
+      </c>
+      <c r="C14" s="242" t="inlineStr">
+        <is>
+          <t>בנק הפועלים</t>
+        </is>
+      </c>
+      <c r="D14" s="242" t="inlineStr">
+        <is>
+          <t>99012</t>
+        </is>
+      </c>
+      <c r="E14" s="242" t="n">
+        <v>350</v>
+      </c>
+      <c r="F14" s="242" t="inlineStr">
+        <is>
+          <t>גואטה מררו אורית</t>
+        </is>
+      </c>
+      <c r="G14" s="242" t="inlineStr">
+        <is>
+          <t>37</t>
+        </is>
+      </c>
+      <c r="H14" s="242" t="inlineStr">
+        <is>
+          <t>חיון</t>
+        </is>
+      </c>
+      <c r="I14" s="242" t="inlineStr"/>
+      <c r="J14" s="242" t="inlineStr">
+        <is>
+          <t>05/2026</t>
+        </is>
+      </c>
+      <c r="K14" s="242" t="inlineStr">
+        <is>
+          <t>fuzzy_name</t>
+        </is>
+      </c>
+      <c r="L14" s="242" t="inlineStr"/>
+      <c r="M14" s="242" t="inlineStr">
+        <is>
+          <t>העברה מאת: גואטה מררו אורית 12-704-000515151 לועד בית חודש מאי</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="16" customHeight="1" s="197">
+      <c r="A15" s="243" t="inlineStr">
+        <is>
+          <t>04/05/2026</t>
+        </is>
+      </c>
+      <c r="B15" s="243" t="inlineStr">
+        <is>
+          <t>הוצאה 💸</t>
+        </is>
+      </c>
+      <c r="C15" s="243" t="inlineStr">
+        <is>
+          <t>העברה דיגיטל</t>
+        </is>
+      </c>
+      <c r="D15" s="243" t="inlineStr">
+        <is>
+          <t>69973</t>
+        </is>
+      </c>
+      <c r="E15" s="243" t="n">
+        <v>900</v>
+      </c>
+      <c r="F15" s="243" t="inlineStr">
+        <is>
+          <t>חלבי כרמי</t>
+        </is>
+      </c>
+      <c r="G15" s="243" t="inlineStr"/>
+      <c r="H15" s="243" t="inlineStr"/>
+      <c r="I15" s="243" t="inlineStr">
+        <is>
+          <t>גינון</t>
+        </is>
+      </c>
+      <c r="J15" s="243" t="inlineStr">
+        <is>
+          <t>05/2026</t>
+        </is>
+      </c>
+      <c r="K15" s="243" t="inlineStr"/>
+      <c r="L15" s="243" t="inlineStr"/>
+      <c r="M15" s="243" t="inlineStr">
+        <is>
+          <t>העברה אל: חלבי כרמי ות 10-981-002104267 גינון</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="16" customHeight="1" s="197">
+      <c r="A16" s="242" t="inlineStr">
+        <is>
+          <t>05/05/2026</t>
+        </is>
+      </c>
+      <c r="B16" s="242" t="inlineStr">
+        <is>
+          <t>הכנסה ✅</t>
+        </is>
+      </c>
+      <c r="C16" s="242" t="inlineStr">
+        <is>
+          <t>בנק דיסקונט</t>
+        </is>
+      </c>
+      <c r="D16" s="242" t="inlineStr">
+        <is>
+          <t>99011</t>
+        </is>
+      </c>
+      <c r="E16" s="242" t="n">
+        <v>320</v>
+      </c>
+      <c r="F16" s="242" t="inlineStr">
+        <is>
+          <t>אסרף אורטל</t>
+        </is>
+      </c>
+      <c r="G16" s="242" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="H16" s="242" t="inlineStr">
+        <is>
+          <t>אסרף אורטל</t>
+        </is>
+      </c>
+      <c r="I16" s="242" t="inlineStr"/>
+      <c r="J16" s="242" t="inlineStr">
+        <is>
+          <t>05/2026</t>
+        </is>
+      </c>
+      <c r="K16" s="242" t="inlineStr">
+        <is>
+          <t>fuzzy_name</t>
+        </is>
+      </c>
+      <c r="L16" s="242" t="inlineStr">
+        <is>
+          <t>⚠️ צפוי ₪350 | בדיקה ידנית</t>
+        </is>
+      </c>
+      <c r="M16" s="242" t="inlineStr">
+        <is>
+          <t>העברה מאת: אסרף אורטל 11-107-081754738</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="16" customHeight="1" s="197">
+      <c r="A17" s="242" t="inlineStr">
+        <is>
+          <t>05/05/2026</t>
+        </is>
+      </c>
+      <c r="B17" s="242" t="inlineStr">
+        <is>
+          <t>הכנסה ✅</t>
+        </is>
+      </c>
+      <c r="C17" s="242" t="inlineStr">
+        <is>
+          <t>בנק אוצר החיל</t>
+        </is>
+      </c>
+      <c r="D17" s="242" t="inlineStr">
+        <is>
+          <t>99014</t>
+        </is>
+      </c>
+      <c r="E17" s="242" t="n">
+        <v>350</v>
+      </c>
+      <c r="F17" s="242" t="inlineStr">
+        <is>
+          <t>כחלון שלו ו/או ח</t>
+        </is>
+      </c>
+      <c r="G17" s="242" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="H17" s="242" t="inlineStr">
+        <is>
+          <t>דון דז'נשבילי</t>
+        </is>
+      </c>
+      <c r="I17" s="242" t="inlineStr"/>
+      <c r="J17" s="242" t="inlineStr">
+        <is>
+          <t>05/2026</t>
+        </is>
+      </c>
+      <c r="K17" s="242" t="inlineStr">
+        <is>
+          <t>apt_hint</t>
+        </is>
+      </c>
+      <c r="L17" s="242" t="inlineStr"/>
+      <c r="M17" s="242" t="inlineStr">
+        <is>
+          <t>העברה מאת: כחלון שלו ו/או ח 14-350-105236062 וועד בית דירה 25 (הערת לקוח)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="16" customHeight="1" s="197">
+      <c r="A18" s="242" t="inlineStr">
+        <is>
+          <t>05/05/2026</t>
+        </is>
+      </c>
+      <c r="B18" s="242" t="inlineStr">
+        <is>
+          <t>הכנסה ✅</t>
+        </is>
+      </c>
+      <c r="C18" s="242" t="inlineStr">
+        <is>
+          <t>הוראת קבע</t>
+        </is>
+      </c>
+      <c r="D18" s="242" t="inlineStr">
+        <is>
+          <t>4789577</t>
+        </is>
+      </c>
+      <c r="E18" s="242" t="n">
+        <v>350</v>
+      </c>
+      <c r="F18" s="242" t="inlineStr">
+        <is>
+          <t>קטרינה שליאק</t>
+        </is>
+      </c>
+      <c r="G18" s="242" t="inlineStr">
+        <is>
+          <t>43</t>
+        </is>
+      </c>
+      <c r="H18" s="242" t="inlineStr">
+        <is>
+          <t>שליאק</t>
+        </is>
+      </c>
+      <c r="I18" s="242" t="inlineStr"/>
+      <c r="J18" s="242" t="inlineStr">
+        <is>
+          <t>05/2026</t>
+        </is>
+      </c>
+      <c r="K18" s="242" t="inlineStr">
+        <is>
+          <t>apt_hint</t>
+        </is>
+      </c>
+      <c r="L18" s="242" t="inlineStr"/>
+      <c r="M18" s="242" t="inlineStr">
+        <is>
+          <t>העברה מאת: קטרינה שליאק 10-838-002943311 דירה 43 משפחת שליאק</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="16" customHeight="1" s="197">
+      <c r="A19" s="242" t="inlineStr">
+        <is>
+          <t>05/05/2026</t>
+        </is>
+      </c>
+      <c r="B19" s="242" t="inlineStr">
+        <is>
+          <t>הכנסה ✅</t>
+        </is>
+      </c>
+      <c r="C19" s="242" t="inlineStr">
+        <is>
+          <t>זיכוי מיידי</t>
+        </is>
+      </c>
+      <c r="D19" s="242" t="inlineStr">
+        <is>
+          <t>106091</t>
+        </is>
+      </c>
+      <c r="E19" s="242" t="n">
+        <v>700</v>
+      </c>
+      <c r="F19" s="242" t="inlineStr">
+        <is>
+          <t>בן לולו נטלי</t>
+        </is>
+      </c>
+      <c r="G19" s="242" t="inlineStr">
+        <is>
+          <t>53</t>
+        </is>
+      </c>
+      <c r="H19" s="242" t="inlineStr">
+        <is>
+          <t>בן לולו</t>
+        </is>
+      </c>
+      <c r="I19" s="242" t="inlineStr"/>
+      <c r="J19" s="242" t="inlineStr">
+        <is>
+          <t>03/2026</t>
+        </is>
+      </c>
+      <c r="K19" s="242" t="inlineStr">
+        <is>
+          <t>fuzzy_name</t>
+        </is>
+      </c>
+      <c r="L19" s="242" t="inlineStr">
+        <is>
+          <t>⚠️ צפוי ₪350 | בדיקה ידנית</t>
+        </is>
+      </c>
+      <c r="M19" s="242" t="inlineStr">
+        <is>
+          <t>העברה מאת: בן לולו נטלי 17-662-098353502 ועד בית מרץ אפריל 62</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="16" customHeight="1" s="197">
+      <c r="A20" s="242" t="inlineStr">
+        <is>
+          <t>06/05/2026</t>
+        </is>
+      </c>
+      <c r="B20" s="242" t="inlineStr">
+        <is>
+          <t>הכנסה ✅</t>
+        </is>
+      </c>
+      <c r="C20" s="242" t="inlineStr">
+        <is>
+          <t>מבנק יהב ס.-י</t>
+        </is>
+      </c>
+      <c r="D20" s="242" t="inlineStr">
+        <is>
+          <t>99004</t>
+        </is>
+      </c>
+      <c r="E20" s="242" t="n">
+        <v>500</v>
+      </c>
+      <c r="F20" s="242" t="inlineStr">
+        <is>
+          <t>אלון ולילך ברכה</t>
+        </is>
+      </c>
+      <c r="G20" s="242" t="inlineStr">
+        <is>
+          <t>54</t>
+        </is>
+      </c>
+      <c r="H20" s="242" t="inlineStr">
+        <is>
+          <t>יוספה אמור</t>
+        </is>
+      </c>
+      <c r="I20" s="242" t="inlineStr"/>
+      <c r="J20" s="242" t="inlineStr">
+        <is>
+          <t>05/2026</t>
+        </is>
+      </c>
+      <c r="K20" s="242" t="inlineStr">
+        <is>
+          <t>fuzzy_name</t>
+        </is>
+      </c>
+      <c r="L20" s="242" t="inlineStr">
+        <is>
+          <t>⚠️ צפוי ₪350 | בדיקה ידנית</t>
+        </is>
+      </c>
+      <c r="M20" s="242" t="inlineStr">
+        <is>
+          <t>העברה מאת: אלון ולילך ברכה 04-140-000085548 38תשלום קופה קטנה דירה</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="16" customHeight="1" s="197">
+      <c r="A21" s="242" t="inlineStr">
+        <is>
+          <t>06/05/2026</t>
+        </is>
+      </c>
+      <c r="B21" s="242" t="inlineStr">
+        <is>
+          <t>הכנסה ✅</t>
+        </is>
+      </c>
+      <c r="C21" s="242" t="inlineStr">
+        <is>
+          <t>הוראת קבע</t>
+        </is>
+      </c>
+      <c r="D21" s="242" t="inlineStr">
+        <is>
+          <t>4870113</t>
+        </is>
+      </c>
+      <c r="E21" s="242" t="n">
+        <v>350</v>
+      </c>
+      <c r="F21" s="242" t="inlineStr">
+        <is>
+          <t>היבה ריזק</t>
+        </is>
+      </c>
+      <c r="G21" s="242" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="H21" s="242" t="inlineStr">
+        <is>
+          <t>ריזק</t>
+        </is>
+      </c>
+      <c r="I21" s="242" t="inlineStr"/>
+      <c r="J21" s="242" t="inlineStr">
+        <is>
+          <t>05/2026</t>
+        </is>
+      </c>
+      <c r="K21" s="242" t="inlineStr">
+        <is>
+          <t>apt_hint</t>
+        </is>
+      </c>
+      <c r="L21" s="242" t="inlineStr"/>
+      <c r="M21" s="242" t="inlineStr">
+        <is>
+          <t>העברה מאת: היבה ריזק 10-840-002040614 ועד בית דירה 32 קומה 7</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="16" customHeight="1" s="197">
+      <c r="A22" s="242" t="inlineStr">
+        <is>
+          <t>08/05/2026</t>
+        </is>
+      </c>
+      <c r="B22" s="242" t="inlineStr">
+        <is>
+          <t>הכנסה ✅</t>
+        </is>
+      </c>
+      <c r="C22" s="242" t="inlineStr">
+        <is>
+          <t>בנק הפועלים</t>
+        </is>
+      </c>
+      <c r="D22" s="242" t="inlineStr">
+        <is>
+          <t>99012</t>
+        </is>
+      </c>
+      <c r="E22" s="242" t="n">
+        <v>350</v>
+      </c>
+      <c r="F22" s="242" t="inlineStr">
+        <is>
+          <t>זאדה הודיה</t>
+        </is>
+      </c>
+      <c r="G22" s="242" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="H22" s="242" t="inlineStr">
+        <is>
+          <t>זאדה הודיה</t>
+        </is>
+      </c>
+      <c r="I22" s="242" t="inlineStr"/>
+      <c r="J22" s="242" t="inlineStr">
+        <is>
+          <t>05/2026</t>
+        </is>
+      </c>
+      <c r="K22" s="242" t="inlineStr">
+        <is>
+          <t>fuzzy_name</t>
+        </is>
+      </c>
+      <c r="L22" s="242" t="inlineStr"/>
+      <c r="M22" s="242" t="inlineStr">
+        <is>
+          <t>העברה מאת: זאדה הודיה 12-703-000404555 תשלום חודשי משפחת זאדה</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="16" customHeight="1" s="197">
+      <c r="A23" s="242" t="inlineStr">
+        <is>
+          <t>08/05/2026</t>
+        </is>
+      </c>
+      <c r="B23" s="242" t="inlineStr">
+        <is>
+          <t>הכנסה ✅</t>
+        </is>
+      </c>
+      <c r="C23" s="242" t="inlineStr">
+        <is>
+          <t>העברה דיגיטל</t>
+        </is>
+      </c>
+      <c r="D23" s="242" t="inlineStr">
+        <is>
+          <t>14334</t>
+        </is>
+      </c>
+      <c r="E23" s="242" t="n">
+        <v>500</v>
+      </c>
+      <c r="F23" s="242" t="inlineStr">
+        <is>
+          <t>טטיאנה סיגל</t>
+        </is>
+      </c>
+      <c r="G23" s="242" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="H23" s="242" t="inlineStr">
+        <is>
+          <t>אלינה סגל</t>
+        </is>
+      </c>
+      <c r="I23" s="242" t="inlineStr"/>
+      <c r="J23" s="242" t="inlineStr">
+        <is>
+          <t>05/2026</t>
+        </is>
+      </c>
+      <c r="K23" s="242" t="inlineStr">
+        <is>
+          <t>fuzzy_name</t>
+        </is>
+      </c>
+      <c r="L23" s="242" t="inlineStr">
+        <is>
+          <t>⚠️ צפוי ₪350 | בדיקה ידנית</t>
+        </is>
+      </c>
+      <c r="M23" s="242" t="inlineStr">
+        <is>
+          <t>העברה מאת: טטיאנה סיגל, 10-882-020472034 תשלום</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="16" customHeight="1" s="197">
+      <c r="A24" s="243" t="inlineStr">
+        <is>
+          <t>10/05/2026</t>
+        </is>
+      </c>
+      <c r="B24" s="243" t="inlineStr">
+        <is>
+          <t>הוצאה 💸</t>
+        </is>
+      </c>
+      <c r="C24" s="243" t="inlineStr">
+        <is>
+          <t>ש.שלמה חברה-י</t>
+        </is>
+      </c>
+      <c r="D24" s="243" t="inlineStr">
+        <is>
+          <t>44855</t>
+        </is>
+      </c>
+      <c r="E24" s="243" t="n">
+        <v>985</v>
+      </c>
+      <c r="F24" s="243" t="inlineStr">
+        <is>
+          <t>ש.שלמה חברה</t>
+        </is>
+      </c>
+      <c r="G24" s="243" t="inlineStr"/>
+      <c r="H24" s="243" t="inlineStr"/>
+      <c r="I24" s="243" t="inlineStr">
+        <is>
+          <t>ביטוח</t>
+        </is>
+      </c>
+      <c r="J24" s="243" t="inlineStr">
+        <is>
+          <t>05/2026</t>
+        </is>
+      </c>
+      <c r="K24" s="243" t="inlineStr"/>
+      <c r="L24" s="243" t="inlineStr"/>
+      <c r="M24" s="243" t="inlineStr"/>
+    </row>
+    <row r="25" ht="16" customHeight="1" s="197">
+      <c r="A25" s="242" t="inlineStr">
+        <is>
+          <t>10/05/2026</t>
+        </is>
+      </c>
+      <c r="B25" s="242" t="inlineStr">
+        <is>
+          <t>הכנסה ✅</t>
+        </is>
+      </c>
+      <c r="C25" s="242" t="inlineStr">
+        <is>
+          <t>בנק דיסקונט</t>
+        </is>
+      </c>
+      <c r="D25" s="242" t="inlineStr">
+        <is>
+          <t>99011</t>
+        </is>
+      </c>
+      <c r="E25" s="242" t="n">
+        <v>350</v>
+      </c>
+      <c r="F25" s="242" t="inlineStr">
+        <is>
+          <t>סימקין טרוסטיאני</t>
+        </is>
+      </c>
+      <c r="G25" s="242" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="H25" s="242" t="inlineStr">
+        <is>
+          <t>סימקין טרוסטיאני</t>
+        </is>
+      </c>
+      <c r="I25" s="242" t="inlineStr"/>
+      <c r="J25" s="242" t="inlineStr">
+        <is>
+          <t>05/2026</t>
+        </is>
+      </c>
+      <c r="K25" s="242" t="inlineStr">
+        <is>
+          <t>apt_hint</t>
+        </is>
+      </c>
+      <c r="L25" s="242" t="inlineStr"/>
+      <c r="M25" s="242" t="inlineStr">
+        <is>
+          <t>העברה מאת: סימקין טרוסטיאני 11-097-132698643 ועד הבית - סימקין דירה 21</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="16" customHeight="1" s="197">
+      <c r="A26" s="242" t="inlineStr">
+        <is>
+          <t>10/05/2026</t>
+        </is>
+      </c>
+      <c r="B26" s="242" t="inlineStr">
+        <is>
+          <t>הכנסה ✅</t>
+        </is>
+      </c>
+      <c r="C26" s="242" t="inlineStr">
+        <is>
+          <t>בנק דיסקונט</t>
+        </is>
+      </c>
+      <c r="D26" s="242" t="inlineStr">
+        <is>
+          <t>99011</t>
+        </is>
+      </c>
+      <c r="E26" s="242" t="n">
+        <v>350</v>
+      </c>
+      <c r="F26" s="242" t="inlineStr">
+        <is>
+          <t>רומנו לינצקי סיו</t>
+        </is>
+      </c>
+      <c r="G26" s="242" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="H26" s="242" t="inlineStr">
+        <is>
+          <t>רומנו לינצקי</t>
+        </is>
+      </c>
+      <c r="I26" s="242" t="inlineStr"/>
+      <c r="J26" s="242" t="inlineStr">
+        <is>
+          <t>05/2026</t>
+        </is>
+      </c>
+      <c r="K26" s="242" t="inlineStr">
+        <is>
+          <t>fuzzy_name</t>
+        </is>
+      </c>
+      <c r="L26" s="242" t="inlineStr"/>
+      <c r="M26" s="242" t="inlineStr">
+        <is>
+          <t>העברה מאת: רומנו לינצקי סיו 11-107-075555974</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="16" customHeight="1" s="197">
+      <c r="A27" s="242" t="inlineStr">
+        <is>
+          <t>10/05/2026</t>
+        </is>
+      </c>
+      <c r="B27" s="242" t="inlineStr">
+        <is>
+          <t>הכנסה ✅</t>
+        </is>
+      </c>
+      <c r="C27" s="242" t="inlineStr">
+        <is>
+          <t>בנק דיסקונט</t>
+        </is>
+      </c>
+      <c r="D27" s="242" t="inlineStr">
+        <is>
+          <t>99011</t>
+        </is>
+      </c>
+      <c r="E27" s="242" t="n">
+        <v>350</v>
+      </c>
+      <c r="F27" s="242" t="inlineStr">
+        <is>
+          <t>שרביט גל,טויזר נ</t>
+        </is>
+      </c>
+      <c r="G27" s="242" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="H27" s="242" t="inlineStr">
+        <is>
+          <t>נוי טויזר</t>
+        </is>
+      </c>
+      <c r="I27" s="242" t="inlineStr"/>
+      <c r="J27" s="242" t="inlineStr">
+        <is>
+          <t>05/2026</t>
+        </is>
+      </c>
+      <c r="K27" s="242" t="inlineStr">
+        <is>
+          <t>apt_hint</t>
+        </is>
+      </c>
+      <c r="L27" s="242" t="inlineStr"/>
+      <c r="M27" s="242" t="inlineStr">
+        <is>
+          <t>העברה מאת: שרביט גל,טויזר נ 11-107-205119303 דירה 60</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="16" customHeight="1" s="197">
+      <c r="A28" s="242" t="inlineStr">
+        <is>
+          <t>10/05/2026</t>
+        </is>
+      </c>
+      <c r="B28" s="242" t="inlineStr">
+        <is>
+          <t>הכנסה ✅</t>
+        </is>
+      </c>
+      <c r="C28" s="242" t="inlineStr">
+        <is>
+          <t>בנק הפועלים</t>
+        </is>
+      </c>
+      <c r="D28" s="242" t="inlineStr">
+        <is>
+          <t>99012</t>
+        </is>
+      </c>
+      <c r="E28" s="242" t="n">
+        <v>350</v>
+      </c>
+      <c r="F28" s="242" t="inlineStr">
+        <is>
+          <t>בייבקוב קו</t>
+        </is>
+      </c>
+      <c r="G28" s="242" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="H28" s="242" t="inlineStr">
+        <is>
+          <t>בייבקוב</t>
+        </is>
+      </c>
+      <c r="I28" s="242" t="inlineStr"/>
+      <c r="J28" s="242" t="inlineStr">
+        <is>
+          <t>05/2026</t>
+        </is>
+      </c>
+      <c r="K28" s="242" t="inlineStr">
+        <is>
+          <t>apt_hint</t>
+        </is>
+      </c>
+      <c r="L28" s="242" t="inlineStr"/>
+      <c r="M28" s="242" t="inlineStr">
+        <is>
+          <t>העברה מאת: בייבקוב קו 12-701-000262613 דירה 9</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="16" customHeight="1" s="197">
+      <c r="A29" s="242" t="inlineStr">
+        <is>
+          <t>10/05/2026</t>
+        </is>
+      </c>
+      <c r="B29" s="242" t="inlineStr">
+        <is>
+          <t>הכנסה ✅</t>
+        </is>
+      </c>
+      <c r="C29" s="242" t="inlineStr">
+        <is>
+          <t>בנק הפועלים</t>
+        </is>
+      </c>
+      <c r="D29" s="242" t="inlineStr">
+        <is>
+          <t>99012</t>
+        </is>
+      </c>
+      <c r="E29" s="242" t="n">
+        <v>350</v>
+      </c>
+      <c r="F29" s="242" t="inlineStr">
+        <is>
+          <t>צ`רניאק בו</t>
+        </is>
+      </c>
+      <c r="G29" s="242" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="H29" s="242" t="inlineStr">
+        <is>
+          <t>צ'רניאק</t>
+        </is>
+      </c>
+      <c r="I29" s="242" t="inlineStr"/>
+      <c r="J29" s="242" t="inlineStr">
+        <is>
+          <t>05/2026</t>
+        </is>
+      </c>
+      <c r="K29" s="242" t="inlineStr">
+        <is>
+          <t>apt_hint</t>
+        </is>
+      </c>
+      <c r="L29" s="242" t="inlineStr"/>
+      <c r="M29" s="242" t="inlineStr">
+        <is>
+          <t>העברה מאת: צ`רניאק בו 12-703-000466089 דירה 44, תשלום ועד</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="16" customHeight="1" s="197">
+      <c r="A30" s="242" t="inlineStr">
+        <is>
+          <t>10/05/2026</t>
+        </is>
+      </c>
+      <c r="B30" s="242" t="inlineStr">
+        <is>
+          <t>הכנסה ✅</t>
+        </is>
+      </c>
+      <c r="C30" s="242" t="inlineStr">
+        <is>
+          <t>בנק הפועלים</t>
+        </is>
+      </c>
+      <c r="D30" s="242" t="inlineStr">
+        <is>
+          <t>99012</t>
+        </is>
+      </c>
+      <c r="E30" s="242" t="n">
+        <v>350</v>
+      </c>
+      <c r="F30" s="242" t="inlineStr">
+        <is>
+          <t>אל איי הנד</t>
+        </is>
+      </c>
+      <c r="G30" s="242" t="inlineStr">
+        <is>
+          <t>57</t>
+        </is>
+      </c>
+      <c r="H30" s="242" t="inlineStr">
+        <is>
+          <t>אל איי</t>
+        </is>
+      </c>
+      <c r="I30" s="242" t="inlineStr"/>
+      <c r="J30" s="242" t="inlineStr">
+        <is>
+          <t>05/2026</t>
+        </is>
+      </c>
+      <c r="K30" s="242" t="inlineStr">
+        <is>
+          <t>apt_hint</t>
+        </is>
+      </c>
+      <c r="L30" s="242" t="inlineStr"/>
+      <c r="M30" s="242" t="inlineStr">
+        <is>
+          <t>העברה מאת: אל איי הנד 12-703-000496840 ועד דירה 57</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="16" customHeight="1" s="197">
+      <c r="A31" s="242" t="inlineStr">
+        <is>
+          <t>10/05/2026</t>
+        </is>
+      </c>
+      <c r="B31" s="242" t="inlineStr">
+        <is>
+          <t>הכנסה ✅</t>
+        </is>
+      </c>
+      <c r="C31" s="242" t="inlineStr">
+        <is>
+          <t>בנק הפועלים</t>
+        </is>
+      </c>
+      <c r="D31" s="242" t="inlineStr">
+        <is>
+          <t>99012</t>
+        </is>
+      </c>
+      <c r="E31" s="242" t="n">
+        <v>350</v>
+      </c>
+      <c r="F31" s="242" t="inlineStr">
+        <is>
+          <t>אסולין יעק</t>
+        </is>
+      </c>
+      <c r="G31" s="242" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="H31" s="242" t="inlineStr">
+        <is>
+          <t>מזרחי</t>
+        </is>
+      </c>
+      <c r="I31" s="242" t="inlineStr"/>
+      <c r="J31" s="242" t="inlineStr">
+        <is>
+          <t>05/2026</t>
+        </is>
+      </c>
+      <c r="K31" s="242" t="inlineStr">
+        <is>
+          <t>fuzzy_name</t>
+        </is>
+      </c>
+      <c r="L31" s="242" t="inlineStr"/>
+      <c r="M31" s="242" t="inlineStr">
+        <is>
+          <t>העברה מאת: אסולין יעק 12-704-000263394 ועד בית</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="16" customHeight="1" s="197">
+      <c r="A32" s="242" t="inlineStr">
+        <is>
+          <t>10/05/2026</t>
+        </is>
+      </c>
+      <c r="B32" s="242" t="inlineStr">
+        <is>
+          <t>הכנסה ✅</t>
+        </is>
+      </c>
+      <c r="C32" s="242" t="inlineStr">
+        <is>
+          <t>בנק הפועלים</t>
+        </is>
+      </c>
+      <c r="D32" s="242" t="inlineStr">
+        <is>
+          <t>99012</t>
+        </is>
+      </c>
+      <c r="E32" s="242" t="n">
+        <v>350</v>
+      </c>
+      <c r="F32" s="242" t="inlineStr">
+        <is>
+          <t>פולונסקי א</t>
+        </is>
+      </c>
+      <c r="G32" s="242" t="inlineStr">
+        <is>
+          <t>52</t>
+        </is>
+      </c>
+      <c r="H32" s="242" t="inlineStr">
+        <is>
+          <t>פולונסקי</t>
+        </is>
+      </c>
+      <c r="I32" s="242" t="inlineStr"/>
+      <c r="J32" s="242" t="inlineStr">
+        <is>
+          <t>05/2026</t>
+        </is>
+      </c>
+      <c r="K32" s="242" t="inlineStr">
+        <is>
+          <t>apt_hint</t>
+        </is>
+      </c>
+      <c r="L32" s="242" t="inlineStr"/>
+      <c r="M32" s="242" t="inlineStr">
+        <is>
+          <t>העברה מאת: פולונסקי א 12-728-000012111 דירה 52</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="16" customHeight="1" s="197">
+      <c r="A33" s="242" t="inlineStr">
+        <is>
+          <t>10/05/2026</t>
+        </is>
+      </c>
+      <c r="B33" s="242" t="inlineStr">
+        <is>
+          <t>הכנסה ✅</t>
+        </is>
+      </c>
+      <c r="C33" s="242" t="inlineStr">
+        <is>
+          <t>בנק אוצר החיל</t>
+        </is>
+      </c>
+      <c r="D33" s="242" t="inlineStr">
+        <is>
+          <t>99014</t>
+        </is>
+      </c>
+      <c r="E33" s="242" t="n">
+        <v>350</v>
+      </c>
+      <c r="F33" s="242" t="inlineStr">
+        <is>
+          <t>כהן אביאל</t>
+        </is>
+      </c>
+      <c r="G33" s="242" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="H33" s="242" t="inlineStr">
+        <is>
+          <t>כהן אביאל</t>
+        </is>
+      </c>
+      <c r="I33" s="242" t="inlineStr"/>
+      <c r="J33" s="242" t="inlineStr">
+        <is>
+          <t>05/2026</t>
+        </is>
+      </c>
+      <c r="K33" s="242" t="inlineStr">
+        <is>
+          <t>fuzzy_name</t>
+        </is>
+      </c>
+      <c r="L33" s="242" t="inlineStr"/>
+      <c r="M33" s="242" t="inlineStr">
+        <is>
+          <t>העברה מאת: כהן אביאל 14-350-000175551 ועד בית</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="16" customHeight="1" s="197">
+      <c r="A34" s="242" t="inlineStr">
+        <is>
+          <t>10/05/2026</t>
+        </is>
+      </c>
+      <c r="B34" s="242" t="inlineStr">
+        <is>
+          <t>הכנסה ✅</t>
+        </is>
+      </c>
+      <c r="C34" s="242" t="inlineStr">
+        <is>
+          <t>בנק אוצר החיל</t>
+        </is>
+      </c>
+      <c r="D34" s="242" t="inlineStr">
+        <is>
+          <t>99014</t>
+        </is>
+      </c>
+      <c r="E34" s="242" t="n">
+        <v>350</v>
+      </c>
+      <c r="F34" s="242" t="inlineStr">
+        <is>
+          <t>זלץ ניר ו/או נט</t>
+        </is>
+      </c>
+      <c r="G34" s="242" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="H34" s="242" t="inlineStr">
+        <is>
+          <t>זלץ</t>
+        </is>
+      </c>
+      <c r="I34" s="242" t="inlineStr"/>
+      <c r="J34" s="242" t="inlineStr">
+        <is>
+          <t>05/2026</t>
+        </is>
+      </c>
+      <c r="K34" s="242" t="inlineStr">
+        <is>
+          <t>fuzzy_name</t>
+        </is>
+      </c>
+      <c r="L34" s="242" t="inlineStr"/>
+      <c r="M34" s="242" t="inlineStr">
+        <is>
+          <t>העברה מאת: זלץ ניר ו/או נט 14-362-105079420 העברה לוועד בית</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="16" customHeight="1" s="197">
+      <c r="A35" s="242" t="inlineStr">
+        <is>
+          <t>10/05/2026</t>
+        </is>
+      </c>
+      <c r="B35" s="242" t="inlineStr">
+        <is>
+          <t>הכנסה ✅</t>
+        </is>
+      </c>
+      <c r="C35" s="242" t="inlineStr">
+        <is>
+          <t>בנק אוצר החיל</t>
+        </is>
+      </c>
+      <c r="D35" s="242" t="inlineStr">
+        <is>
+          <t>99014</t>
+        </is>
+      </c>
+      <c r="E35" s="242" t="n">
+        <v>350</v>
+      </c>
+      <c r="F35" s="242" t="inlineStr">
+        <is>
+          <t>איטח ענת ו/או רפ</t>
+        </is>
+      </c>
+      <c r="G35" s="242" t="inlineStr">
+        <is>
+          <t>59</t>
+        </is>
+      </c>
+      <c r="H35" s="242" t="inlineStr">
+        <is>
+          <t>איטח ענת</t>
+        </is>
+      </c>
+      <c r="I35" s="242" t="inlineStr"/>
+      <c r="J35" s="242" t="inlineStr">
+        <is>
+          <t>05/2026</t>
+        </is>
+      </c>
+      <c r="K35" s="242" t="inlineStr">
+        <is>
+          <t>fuzzy_name</t>
+        </is>
+      </c>
+      <c r="L35" s="242" t="inlineStr"/>
+      <c r="M35" s="242" t="inlineStr">
+        <is>
+          <t>העברה מאת: איטח ענת ו/או רפ 14-362-000321489 איטח ענת ורפי</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="16" customHeight="1" s="197">
+      <c r="A36" s="242" t="inlineStr">
+        <is>
+          <t>10/05/2026</t>
+        </is>
+      </c>
+      <c r="B36" s="242" t="inlineStr">
+        <is>
+          <t>הכנסה ✅</t>
+        </is>
+      </c>
+      <c r="C36" s="242" t="inlineStr">
+        <is>
+          <t>בנק מזרחי</t>
+        </is>
+      </c>
+      <c r="D36" s="242" t="inlineStr">
+        <is>
+          <t>99020</t>
+        </is>
+      </c>
+      <c r="E36" s="242" t="n">
+        <v>350</v>
+      </c>
+      <c r="F36" s="242" t="inlineStr">
+        <is>
+          <t>וולמיר רות ואלכס</t>
+        </is>
+      </c>
+      <c r="G36" s="242" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="H36" s="242" t="inlineStr">
+        <is>
+          <t>וולמיר רות</t>
+        </is>
+      </c>
+      <c r="I36" s="242" t="inlineStr"/>
+      <c r="J36" s="242" t="inlineStr">
+        <is>
+          <t>05/2026</t>
+        </is>
+      </c>
+      <c r="K36" s="242" t="inlineStr">
+        <is>
+          <t>apt_hint</t>
+        </is>
+      </c>
+      <c r="L36" s="242" t="inlineStr"/>
+      <c r="M36" s="242" t="inlineStr">
+        <is>
+          <t>העברה מאת: וולמיר רות ואלכס 20-441-000075228 עבור דירה 7</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="16" customHeight="1" s="197">
+      <c r="A37" s="242" t="inlineStr">
+        <is>
+          <t>10/05/2026</t>
+        </is>
+      </c>
+      <c r="B37" s="242" t="inlineStr">
+        <is>
+          <t>הכנסה ✅</t>
+        </is>
+      </c>
+      <c r="C37" s="242" t="inlineStr">
+        <is>
+          <t>הוראת קבע</t>
+        </is>
+      </c>
+      <c r="D37" s="242" t="inlineStr">
+        <is>
+          <t>4512636</t>
+        </is>
+      </c>
+      <c r="E37" s="242" t="n">
+        <v>350</v>
+      </c>
+      <c r="F37" s="242" t="inlineStr">
+        <is>
+          <t>קוטיגרו מיכאל</t>
+        </is>
+      </c>
+      <c r="G37" s="242" t="inlineStr">
+        <is>
+          <t>46</t>
+        </is>
+      </c>
+      <c r="H37" s="242" t="inlineStr">
+        <is>
+          <t>קוטיגרו</t>
+        </is>
+      </c>
+      <c r="I37" s="242" t="inlineStr"/>
+      <c r="J37" s="242" t="inlineStr">
+        <is>
+          <t>05/2026</t>
+        </is>
+      </c>
+      <c r="K37" s="242" t="inlineStr">
+        <is>
+          <t>fuzzy_name</t>
+        </is>
+      </c>
+      <c r="L37" s="242" t="inlineStr"/>
+      <c r="M37" s="242" t="inlineStr">
+        <is>
+          <t>העברה מאת: קוטיגרו מיכאל 10-948-057374636 תשלום</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="16" customHeight="1" s="197">
+      <c r="A38" s="242" t="inlineStr">
+        <is>
+          <t>10/05/2026</t>
+        </is>
+      </c>
+      <c r="B38" s="242" t="inlineStr">
+        <is>
+          <t>הכנסה ✅</t>
+        </is>
+      </c>
+      <c r="C38" s="242" t="inlineStr">
+        <is>
+          <t>הוראת קבע</t>
+        </is>
+      </c>
+      <c r="D38" s="242" t="inlineStr">
+        <is>
+          <t>4763312</t>
+        </is>
+      </c>
+      <c r="E38" s="242" t="n">
+        <v>350</v>
+      </c>
+      <c r="F38" s="242" t="inlineStr">
+        <is>
+          <t>יוספה אמור, בנימ</t>
+        </is>
+      </c>
+      <c r="G38" s="242" t="inlineStr">
+        <is>
+          <t>54</t>
+        </is>
+      </c>
+      <c r="H38" s="242" t="inlineStr">
+        <is>
+          <t>יוספה אמור</t>
+        </is>
+      </c>
+      <c r="I38" s="242" t="inlineStr"/>
+      <c r="J38" s="242" t="inlineStr">
+        <is>
+          <t>05/2026</t>
+        </is>
+      </c>
+      <c r="K38" s="242" t="inlineStr">
+        <is>
+          <t>fuzzy_name</t>
+        </is>
+      </c>
+      <c r="L38" s="242" t="inlineStr"/>
+      <c r="M38" s="242" t="inlineStr">
+        <is>
+          <t>העברה מאת: יוספה אמור, בנימ 10-885-000271821 תשלום בהוראת קבע</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="16" customHeight="1" s="197">
+      <c r="A39" s="242" t="inlineStr">
+        <is>
+          <t>10/05/2026</t>
+        </is>
+      </c>
+      <c r="B39" s="242" t="inlineStr">
+        <is>
+          <t>הכנסה ✅</t>
+        </is>
+      </c>
+      <c r="C39" s="242" t="inlineStr">
+        <is>
+          <t>הוראת קבע</t>
+        </is>
+      </c>
+      <c r="D39" s="242" t="inlineStr">
+        <is>
+          <t>4875354</t>
+        </is>
+      </c>
+      <c r="E39" s="242" t="n">
+        <v>350</v>
+      </c>
+      <c r="F39" s="242" t="inlineStr">
+        <is>
+          <t>בר ברקת ישראלי</t>
+        </is>
+      </c>
+      <c r="G39" s="242" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="H39" s="242" t="inlineStr">
+        <is>
+          <t>ישראלי</t>
+        </is>
+      </c>
+      <c r="I39" s="242" t="inlineStr"/>
+      <c r="J39" s="242" t="inlineStr">
+        <is>
+          <t>05/2026</t>
+        </is>
+      </c>
+      <c r="K39" s="242" t="inlineStr">
+        <is>
+          <t>apt_hint</t>
+        </is>
+      </c>
+      <c r="L39" s="242" t="inlineStr"/>
+      <c r="M39" s="242" t="inlineStr">
+        <is>
+          <t>העברה מאת: בר ברקת ישראלי, 10-716-002056289 ועד בית דירה 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="16" customHeight="1" s="197">
+      <c r="A40" s="242" t="inlineStr">
+        <is>
+          <t>10/05/2026</t>
+        </is>
+      </c>
+      <c r="B40" s="242" t="inlineStr">
+        <is>
+          <t>הכנסה ✅</t>
+        </is>
+      </c>
+      <c r="C40" s="242" t="inlineStr">
+        <is>
+          <t>הוראת קבע</t>
+        </is>
+      </c>
+      <c r="D40" s="242" t="inlineStr">
+        <is>
+          <t>4883868</t>
+        </is>
+      </c>
+      <c r="E40" s="242" t="n">
+        <v>350</v>
+      </c>
+      <c r="F40" s="242" t="inlineStr">
+        <is>
+          <t>לאוניד שכטמן</t>
+        </is>
+      </c>
+      <c r="G40" s="242" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="H40" s="242" t="inlineStr">
+        <is>
+          <t>שכטמן</t>
+        </is>
+      </c>
+      <c r="I40" s="242" t="inlineStr"/>
+      <c r="J40" s="242" t="inlineStr">
+        <is>
+          <t>05/2026</t>
+        </is>
+      </c>
+      <c r="K40" s="242" t="inlineStr">
+        <is>
+          <t>fuzzy_name</t>
+        </is>
+      </c>
+      <c r="L40" s="242" t="inlineStr"/>
+      <c r="M40" s="242" t="inlineStr">
+        <is>
+          <t>העברה מאת: לאוניד שכטמן 10-705-012376080 ועד בית</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="16" customHeight="1" s="197">
+      <c r="A41" s="242" t="inlineStr">
+        <is>
+          <t>10/05/2026</t>
+        </is>
+      </c>
+      <c r="B41" s="242" t="inlineStr">
+        <is>
+          <t>הכנסה ✅</t>
+        </is>
+      </c>
+      <c r="C41" s="242" t="inlineStr">
+        <is>
+          <t>הוראת קבע</t>
+        </is>
+      </c>
+      <c r="D41" s="242" t="inlineStr">
+        <is>
+          <t>4899758</t>
+        </is>
+      </c>
+      <c r="E41" s="242" t="n">
+        <v>350</v>
+      </c>
+      <c r="F41" s="242" t="inlineStr">
+        <is>
+          <t>וולושין אלכסנדר</t>
+        </is>
+      </c>
+      <c r="G41" s="242" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="H41" s="242" t="inlineStr">
+        <is>
+          <t>וולושין</t>
+        </is>
+      </c>
+      <c r="I41" s="242" t="inlineStr"/>
+      <c r="J41" s="242" t="inlineStr">
+        <is>
+          <t>05/2026</t>
+        </is>
+      </c>
+      <c r="K41" s="242" t="inlineStr">
+        <is>
+          <t>fuzzy_name</t>
+        </is>
+      </c>
+      <c r="L41" s="242" t="inlineStr"/>
+      <c r="M41" s="242" t="inlineStr">
+        <is>
+          <t>העברה מאת: וולושין אלכסנדר 10-879-057984481 ועד בית</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="16" customHeight="1" s="197">
+      <c r="A42" s="242" t="inlineStr">
+        <is>
+          <t>10/05/2026</t>
+        </is>
+      </c>
+      <c r="B42" s="242" t="inlineStr">
+        <is>
+          <t>הכנסה ✅</t>
+        </is>
+      </c>
+      <c r="C42" s="242" t="inlineStr">
+        <is>
+          <t>הוראת קבע</t>
+        </is>
+      </c>
+      <c r="D42" s="242" t="inlineStr">
+        <is>
+          <t>4908474</t>
+        </is>
+      </c>
+      <c r="E42" s="242" t="n">
+        <v>350</v>
+      </c>
+      <c r="F42" s="242" t="inlineStr">
+        <is>
+          <t>מנגסטה יטמין</t>
+        </is>
+      </c>
+      <c r="G42" s="242" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="H42" s="242" t="inlineStr">
+        <is>
+          <t>לב ארי</t>
+        </is>
+      </c>
+      <c r="I42" s="242" t="inlineStr"/>
+      <c r="J42" s="242" t="inlineStr">
+        <is>
+          <t>05/2026</t>
+        </is>
+      </c>
+      <c r="K42" s="242" t="inlineStr">
+        <is>
+          <t>apt_hint</t>
+        </is>
+      </c>
+      <c r="L42" s="242" t="inlineStr"/>
+      <c r="M42" s="242" t="inlineStr">
+        <is>
+          <t>העברה מאת: מנגסטה יטמין 10-885-001146229 דירה 8</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="16" customHeight="1" s="197">
+      <c r="A43" s="243" t="inlineStr">
+        <is>
+          <t>10/05/2026</t>
+        </is>
+      </c>
+      <c r="B43" s="243" t="inlineStr">
+        <is>
+          <t>הוצאה 💸</t>
+        </is>
+      </c>
+      <c r="C43" s="243" t="inlineStr">
+        <is>
+          <t>הוראת קבע</t>
+        </is>
+      </c>
+      <c r="D43" s="243" t="inlineStr">
+        <is>
+          <t>4932477</t>
+        </is>
+      </c>
+      <c r="E43" s="243" t="n">
+        <v>7500</v>
+      </c>
+      <c r="F43" s="243" t="inlineStr">
+        <is>
+          <t>יניב אחזקות</t>
+        </is>
+      </c>
+      <c r="G43" s="243" t="inlineStr"/>
+      <c r="H43" s="243" t="inlineStr"/>
+      <c r="I43" s="243" t="inlineStr">
+        <is>
+          <t>יניב אחזקות</t>
+        </is>
+      </c>
+      <c r="J43" s="243" t="inlineStr">
+        <is>
+          <t>05/2026</t>
+        </is>
+      </c>
+      <c r="K43" s="243" t="inlineStr"/>
+      <c r="L43" s="243" t="inlineStr"/>
+      <c r="M43" s="243" t="inlineStr">
+        <is>
+          <t>העברה ל: גל אנתבי 20-505-00159972 תאריך סיום: 09.12.2027 ניקיון האגמית 7</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>